<commit_message>
unfinished ocb with parts list
</commit_message>
<xml_diff>
--- a/Electrical/PCB V2 ( 26 Nov)/L1/Parts List L1 V2.xlsx
+++ b/Electrical/PCB V2 ( 26 Nov)/L1/Parts List L1 V2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4ad0bf7e61e147d2/Documents/GitHub/robocup2025/Electrical/PCB v1/L1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4ad0bf7e61e147d2/Documents/GitHub/robocup2025/Electrical/PCB V2 ( 26 Nov)/L1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="11_F25DC773A252ABDACC1048BDC11F63425BDE58E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B28DA38D-9404-4BCF-AD26-617C4EDC1019}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="11_F25DC773A252ABDACC1048BDC11F63425BDE58E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EDE064B-E288-48F3-9B8F-A500479F03B8}"/>
   <bookViews>
-    <workbookView xWindow="10958" yWindow="0" windowWidth="11205" windowHeight="13163" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22276" windowHeight="13276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t xml:space="preserve">Parts list </t>
   </si>
@@ -83,30 +83,18 @@
     <t>LEDS</t>
   </si>
   <si>
-    <t>SM0603UYC</t>
-  </si>
-  <si>
     <t>0.8 x 0.6 x 1.7</t>
   </si>
   <si>
     <t>1.6mm x 0.8mm x 0.6 mm</t>
   </si>
   <si>
-    <t>ESP32-WROOM-32D (16MB)</t>
-  </si>
-  <si>
-    <t>25.5 X 18 X 3.2</t>
-  </si>
-  <si>
     <t>Muxes</t>
   </si>
   <si>
     <t>CD74HC4067SM</t>
   </si>
   <si>
-    <t>https://www.snapeda.com/parts/ESP32-WROOM-32D-N4/Espressif%20Systems/datasheet/</t>
-  </si>
-  <si>
     <t>https://www.snapeda.com/parts/CD74HC4067SM96G4/Texas%20Instruments/datasheet/</t>
   </si>
   <si>
@@ -117,6 +105,27 @@
   </si>
   <si>
     <t>0.05( actl 0 cos lab have)</t>
+  </si>
+  <si>
+    <t>not required as in lab</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>not required to buy</t>
+  </si>
+  <si>
+    <t>to buy</t>
+  </si>
+  <si>
+    <t>lab</t>
+  </si>
+  <si>
+    <t>kicad smd thingy</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> XIAO 102010428</t>
   </si>
 </sst>
 </file>
@@ -456,127 +465,136 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.59765625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="102.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="102.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>5</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>7</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>6</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="1">
-        <v>3</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>22</v>
-      </c>
+      <c r="G4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>10</v>
       </c>
-      <c r="E5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="1">
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="1">
         <v>0.05</v>
       </c>
-      <c r="G5" s="3" t="str">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_1806131537_Everlight-Elec-ALS-PT19-315C-L177-TR8_C146233.pdf")</f>
-        <v>https://www.lcsc.com/datasheet/lcsc_datasheet_1806131537_Everlight-Elec-ALS-PT19-315C-L177-TR8_C146233.pdf</v>
-      </c>
+      <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
         <v>17</v>
       </c>
-      <c r="F6" t="s">
+      <c r="B7" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" t="s">
+      <c r="G7" t="s">
         <v>21</v>
       </c>
-      <c r="E7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" t="s">
-        <v>23</v>
+      <c r="H7" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>